<commit_message>
Enhance sensitivity analysis scripts and update .gitignore
- Updated .gitignore to include sweep_results_*.xlsx files.
- Modified DoE_main_sensitivity.m to support ICE powertrain in addition to Hybrid and BEV.
- Expanded run_sensitivity_pipeline.py to include ICE powertrain handling, updated argument parsing, and adjusted default values for powertrain selection.
- Added new sensitivity analysis scripts for ICE powertrain.
- Updated various sweep result files for G2 and G4 tasks.
</commit_message>
<xml_diff>
--- a/Data_Analysis/Sensitivity analysis/Hybrid/sweep_results_hybrid_G1_task019.xlsx
+++ b/Data_Analysis/Sensitivity analysis/Hybrid/sweep_results_hybrid_G1_task019.xlsx
@@ -100,7 +100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.85546875" customWidth="true"/>
@@ -339,6 +339,50 @@
         <v>5.2599326055393023</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>75</v>
+      </c>
+      <c r="B6" s="0">
+        <v>185</v>
+      </c>
+      <c r="C6" s="0">
+        <v>75</v>
+      </c>
+      <c r="D6" s="0">
+        <v>94.182006401943326</v>
+      </c>
+      <c r="E6" s="0">
+        <v>473.78500000000003</v>
+      </c>
+      <c r="F6" s="0">
+        <v>155.45361751329582</v>
+      </c>
+      <c r="G6" s="0">
+        <v>3377.5179472032778</v>
+      </c>
+      <c r="H6" s="0">
+        <v>-800.85213932780835</v>
+      </c>
+      <c r="I6" s="0">
+        <v>5.2300000000000004</v>
+      </c>
+      <c r="J6" s="0">
+        <v>15.41</v>
+      </c>
+      <c r="K6" s="0">
+        <v>2.5</v>
+      </c>
+      <c r="L6" s="0">
+        <v>3.5699999999999998</v>
+      </c>
+      <c r="M6" s="0">
+        <v>286.20122975094102</v>
+      </c>
+      <c r="N6" s="0">
+        <v>5.2599326055393023</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>